<commit_message>
feat: Door 1차 완성
- 문 잠금 해제 시 삭제
- 문 열리는 에셋 적용 필요 여부 확인 후 애니메이션 넣을지 판단
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Door.xlsx
+++ b/JsonConverter/ExcelFiles/Door.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>데이터 Id</t>
   </si>
@@ -22,6 +22,14 @@
     <t>오브젝트 설명</t>
   </si>
   <si>
+    <t>잠금해제 도구 데이터 ID
+(해제 리스트)</t>
+  </si>
+  <si>
+    <t>강제 개방 시 줄어드는 시간
+(키사용, 락픽사용)</t>
+  </si>
+  <si>
     <t>잠금 여부</t>
   </si>
   <si>
@@ -31,6 +39,12 @@
     <t>string</t>
   </si>
   <si>
+    <t>string[]</t>
+  </si>
+  <si>
+    <t>float[]</t>
+  </si>
+  <si>
     <t>bool</t>
   </si>
   <si>
@@ -43,7 +57,13 @@
     <t>DoorComment</t>
   </si>
   <si>
-    <t>IsLock</t>
+    <t>DoorRequiresToolIdList</t>
+  </si>
+  <si>
+    <t>DoorTimeReductionAmountList</t>
+  </si>
+  <si>
+    <t>IsDisarm</t>
   </si>
   <si>
     <t>DoorMeshPrefabPath</t>
@@ -52,22 +72,25 @@
     <t>Door_01</t>
   </si>
   <si>
-    <t>문</t>
-  </si>
-  <si>
-    <t>문이다. 잠금장치가 존재하지 않아 그냥 열 수 있을거 같다.</t>
+    <t>잠긴 문</t>
+  </si>
+  <si>
+    <t>문이다. 잠금장치가 존재하여 도구를 사용해야 열 수 있을거 같다.</t>
+  </si>
+  <si>
+    <t>0, 10</t>
   </si>
   <si>
     <t>false</t>
   </si>
   <si>
-    <t>Door_02</t>
-  </si>
-  <si>
-    <t>잠긴 문</t>
-  </si>
-  <si>
-    <t>문이다. 잠금장치가 존재하여 도구를 사용해야 열 수 있을거 같다.</t>
+    <t>Assets/03_Prefabs/Object/Door_Mesh</t>
+  </si>
+  <si>
+    <t>Door_Test_Opened</t>
+  </si>
+  <si>
+    <t>철문(잠김)</t>
   </si>
   <si>
     <t>true</t>
@@ -77,7 +100,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -91,6 +114,10 @@
     <font>
       <color rgb="FF000000"/>
       <name val="&quot;맑은 고딕&quot;"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="4">
@@ -240,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -249,6 +276,9 @@
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
@@ -259,6 +289,9 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -268,28 +301,28 @@
     <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
     <xf borderId="9" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="11" fillId="2" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="11" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="11" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -509,9 +542,11 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="37.88"/>
-    <col customWidth="1" min="4" max="4" width="14.25"/>
-    <col customWidth="1" min="5" max="5" width="15.38"/>
+    <col customWidth="1" min="1" max="1" width="15.5"/>
+    <col customWidth="1" min="3" max="3" width="20.5"/>
+    <col customWidth="1" min="4" max="4" width="20.0"/>
+    <col customWidth="1" min="5" max="6" width="14.25"/>
+    <col customWidth="1" min="7" max="7" width="15.38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,97 +559,109 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>5</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="9" t="s">
+      <c r="A3" s="9" t="s">
         <v>11</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="13"/>
+      <c r="A4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="15"/>
+      <c r="E4" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>16</v>
+      <c r="A5" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="15"/>
+        <v>25</v>
+      </c>
+      <c r="C5" s="14"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="18"/>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
+      <c r="A6" s="6"/>
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
-      <c r="D6" s="12"/>
+      <c r="D6" s="15"/>
       <c r="E6" s="16"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="16"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="18"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>